<commit_message>
Add run report and log clearing
</commit_message>
<xml_diff>
--- a/templates/Trial Balance_template.xlsx
+++ b/templates/Trial Balance_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/richardpalenik/Dropbox/python-development/GenAI/ecos/trial_balance/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55172CB2-1A30-AE4C-AC52-11152B0A5557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB69C62-C1F7-BD48-8D80-9896ED283EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="10220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trial Balance_30.11.2025" sheetId="1" r:id="rId1"/>

</xml_diff>